<commit_message>
Update labeler guide for the UNI-300VA line
- Rebuild the guide around the NJM UNI-300VA with the Videojet DataFlex
  6320 coder and Optel vision, keeping only common alarms an operator
  can clear (inspection, labels, ribbon, jams, guards, E-stop)
- Show which screen each alarm appears on and add a call-your-lead note
- Size rows for wrapped text so steps aren't cut off
- Rename the file to Error Code Guide - UNI-300VA Labeler.xlsx
- App: same alarms as the example, note row and matching layout in the
  Excel download

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Np6FjV33ZtJzjSs2EYKhw9
</commit_message>
<xml_diff>
--- a/Error Code Guide - Blank.xlsx
+++ b/Error Code Guide - Blank.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,7 +31,7 @@
       <name val="Aptos Narrow"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="24"/>
+      <sz val="22"/>
     </font>
     <font>
       <name val="Aptos Narrow"/>
@@ -56,8 +56,14 @@
       <color rgb="00222222"/>
       <sz val="13"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="009C1C1C"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +83,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEBD8"/>
       </patternFill>
     </fill>
   </fills>
@@ -111,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -133,6 +144,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -529,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -649,9 +663,17 @@
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
     </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>NOTE: If these steps don't fix it, or the same error keeps coming back, stop the line and call your lead or mechanic. Do not change machine settings.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:B2"/>
+    <mergeCell ref="A21:C21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Add pictures to the error code guide app
- Picture column and a machine picture (own Machine Map tab in Excel)
- Marking tool: box, circle, arrow, label, dim the rest
- Pictures go into the Excel download and come back with Open Excel
- Photos are kept in the browser's database and synced by cloud save as
  locked files in a second gist, uploaded once
- UNI-300VA example and guide: real screen wording (VISION INSPECTION
  FAIL, RESET ALARM) and the Optel Unexpected Product warning
- Blank template gets a PICTURE column

No machine photos are included in the repository.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Np6FjV33ZtJzjSs2EYKhw9
</commit_message>
<xml_diff>
--- a/Error Code Guide - Blank.xlsx
+++ b/Error Code Guide - Blank.xlsx
@@ -228,7 +228,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>2</col>
+      <col>3</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
@@ -543,12 +543,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -558,10 +559,12 @@
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
     </row>
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="n"/>
       <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -587,81 +590,101 @@
           <t>STEPS TO FIX</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="90" customHeight="1">
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>PICTURE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="150" customHeight="1">
       <c r="A5" s="6" t="n"/>
       <c r="B5" s="7" t="n"/>
       <c r="C5" s="7" t="n"/>
-    </row>
-    <row r="6" ht="90" customHeight="1">
+      <c r="D5" s="7" t="n"/>
+    </row>
+    <row r="6" ht="150" customHeight="1">
       <c r="A6" s="8" t="n"/>
       <c r="B6" s="9" t="n"/>
       <c r="C6" s="9" t="n"/>
-    </row>
-    <row r="7" ht="90" customHeight="1">
+      <c r="D6" s="9" t="n"/>
+    </row>
+    <row r="7" ht="150" customHeight="1">
       <c r="A7" s="6" t="n"/>
       <c r="B7" s="7" t="n"/>
       <c r="C7" s="7" t="n"/>
-    </row>
-    <row r="8" ht="90" customHeight="1">
+      <c r="D7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="150" customHeight="1">
       <c r="A8" s="8" t="n"/>
       <c r="B8" s="9" t="n"/>
       <c r="C8" s="9" t="n"/>
-    </row>
-    <row r="9" ht="90" customHeight="1">
+      <c r="D8" s="9" t="n"/>
+    </row>
+    <row r="9" ht="150" customHeight="1">
       <c r="A9" s="6" t="n"/>
       <c r="B9" s="7" t="n"/>
       <c r="C9" s="7" t="n"/>
-    </row>
-    <row r="10" ht="90" customHeight="1">
+      <c r="D9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="150" customHeight="1">
       <c r="A10" s="8" t="n"/>
       <c r="B10" s="9" t="n"/>
       <c r="C10" s="9" t="n"/>
-    </row>
-    <row r="11" ht="90" customHeight="1">
+      <c r="D10" s="9" t="n"/>
+    </row>
+    <row r="11" ht="150" customHeight="1">
       <c r="A11" s="6" t="n"/>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="7" t="n"/>
-    </row>
-    <row r="12" ht="90" customHeight="1">
+      <c r="D11" s="7" t="n"/>
+    </row>
+    <row r="12" ht="150" customHeight="1">
       <c r="A12" s="8" t="n"/>
       <c r="B12" s="9" t="n"/>
       <c r="C12" s="9" t="n"/>
-    </row>
-    <row r="13" ht="90" customHeight="1">
+      <c r="D12" s="9" t="n"/>
+    </row>
+    <row r="13" ht="150" customHeight="1">
       <c r="A13" s="6" t="n"/>
       <c r="B13" s="7" t="n"/>
       <c r="C13" s="7" t="n"/>
-    </row>
-    <row r="14" ht="90" customHeight="1">
+      <c r="D13" s="7" t="n"/>
+    </row>
+    <row r="14" ht="150" customHeight="1">
       <c r="A14" s="8" t="n"/>
       <c r="B14" s="9" t="n"/>
       <c r="C14" s="9" t="n"/>
-    </row>
-    <row r="15" ht="90" customHeight="1">
+      <c r="D14" s="9" t="n"/>
+    </row>
+    <row r="15" ht="150" customHeight="1">
       <c r="A15" s="6" t="n"/>
       <c r="B15" s="7" t="n"/>
       <c r="C15" s="7" t="n"/>
-    </row>
-    <row r="16" ht="90" customHeight="1">
+      <c r="D15" s="7" t="n"/>
+    </row>
+    <row r="16" ht="150" customHeight="1">
       <c r="A16" s="8" t="n"/>
       <c r="B16" s="9" t="n"/>
       <c r="C16" s="9" t="n"/>
-    </row>
-    <row r="17" ht="90" customHeight="1">
+      <c r="D16" s="9" t="n"/>
+    </row>
+    <row r="17" ht="150" customHeight="1">
       <c r="A17" s="6" t="n"/>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
+      <c r="D17" s="7" t="n"/>
+    </row>
+    <row r="18" ht="150" customHeight="1">
       <c r="A18" s="8" t="n"/>
       <c r="B18" s="9" t="n"/>
       <c r="C18" s="9" t="n"/>
-    </row>
-    <row r="19" ht="90" customHeight="1">
+      <c r="D18" s="9" t="n"/>
+    </row>
+    <row r="19" ht="150" customHeight="1">
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
     </row>
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -672,8 +695,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="A21:D21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Redesign the Excel guide banner, keeping the Pharmavite logo
- Gold accent strip, navy title block with OPERATOR'S TROUBLESHOOTING
  GUIDE over the machine name, and the logo centered in its own panel
- How-to line with the date the guide was made; gold edge on each error
  code and a red edge on the note
- Same banner on the Machine Map tab and the blank template (which gets
  Machine / Line / Updated blanks)
- Open Excel reads the machine name from the new banner, older titles
  and 'Operator's Troubleshooting Guide' titles

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Np6FjV33ZtJzjSs2EYKhw9
</commit_message>
<xml_diff>
--- a/Error Code Guide - Blank.xlsx
+++ b/Error Code Guide - Blank.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Error Codes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Error Codes'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Error Codes'!$6:$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -30,20 +30,21 @@
     <font>
       <name val="Aptos Narrow"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="22"/>
+      <color rgb="001F3A4D"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="006B7B8C"/>
+      <sz val="10.5"/>
     </font>
     <font>
       <name val="Aptos Narrow"/>
       <b val="1"/>
       <color rgb="001F3A4D"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <b val="1"/>
-      <color rgb="001F3A4D"/>
-      <sz val="12"/>
     </font>
     <font>
       <name val="Aptos Narrow"/>
@@ -63,7 +64,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -72,12 +73,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3A4D"/>
+        <fgColor rgb="00F6B53B"/>
       </patternFill>
     </fill>
     <fill>
+      <gradientFill type="linear">
+        <stop position="0">
+          <color rgb="001F3A4D"/>
+        </stop>
+        <stop position="1">
+          <color rgb="002F5878"/>
+        </stop>
+      </gradientFill>
+    </fill>
+    <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F6B53B"/>
+        <fgColor rgb="00E9EFF5"/>
       </patternFill>
     </fill>
     <fill>
@@ -91,13 +102,18 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D0D7DE"/>
+      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -114,38 +130,57 @@
       </bottom>
     </border>
     <border>
+      <left style="thick">
+        <color rgb="00F6B53B"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D7DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D7DE"/>
+      </top>
       <bottom style="thin">
-        <color rgb="001F3A4D"/>
+        <color rgb="00D0D7DE"/>
       </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00C62828"/>
+      </left>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -229,11 +264,11 @@
   <oneCellAnchor>
     <from>
       <col>3</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
+      <colOff>1647825</colOff>
+      <row>1</row>
+      <rowOff>66675</rowOff>
     </from>
-    <ext cx="666750" cy="762000"/>
+    <ext cx="609600" cy="704850"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -543,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -552,151 +587,177 @@
     <col width="58" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="7" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ERROR CODE GUIDE</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="00F6B53B"/>
+              <sz val="11"/>
+            </rPr>
+            <t>OPERATOR'S TROUBLESHOOTING GUIDE</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="00FFFFFF"/>
+              <sz val="26"/>
+            </rPr>
+            <t xml:space="preserve">
+ERROR CODE GUIDE</t>
+          </r>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="D2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="36" customHeight="1"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>MACHINE:</t>
+          <t>MACHINE: ________________________________          LINE: ____________</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n"/>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>UPDATED: ________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="6" customHeight="1"/>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>ERROR CODE</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>POSSIBLE PROBLEM</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>STEPS TO FIX</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>PICTURE</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="150" customHeight="1">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-    </row>
-    <row r="6" ht="150" customHeight="1">
-      <c r="A6" s="8" t="n"/>
-      <c r="B6" s="9" t="n"/>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
-    </row>
     <row r="7" ht="150" customHeight="1">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
     </row>
     <row r="8" ht="150" customHeight="1">
-      <c r="A8" s="8" t="n"/>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
+      <c r="A8" s="9" t="n"/>
+      <c r="B8" s="10" t="n"/>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="10" t="n"/>
     </row>
     <row r="9" ht="150" customHeight="1">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
     </row>
     <row r="10" ht="150" customHeight="1">
-      <c r="A10" s="8" t="n"/>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
+      <c r="A10" s="9" t="n"/>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
     </row>
     <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
     </row>
     <row r="12" ht="150" customHeight="1">
-      <c r="A12" s="8" t="n"/>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
+      <c r="A12" s="9" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
     </row>
     <row r="13" ht="150" customHeight="1">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
     </row>
     <row r="14" ht="150" customHeight="1">
-      <c r="A14" s="8" t="n"/>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
+      <c r="A14" s="9" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
     </row>
     <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
     </row>
     <row r="16" ht="150" customHeight="1">
-      <c r="A16" s="8" t="n"/>
-      <c r="B16" s="9" t="n"/>
-      <c r="C16" s="9" t="n"/>
-      <c r="D16" s="9" t="n"/>
+      <c r="A16" s="9" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
     </row>
     <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
+      <c r="A17" s="7" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
     </row>
     <row r="18" ht="150" customHeight="1">
-      <c r="A18" s="8" t="n"/>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
+      <c r="A18" s="9" t="n"/>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
     </row>
     <row r="19" ht="150" customHeight="1">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-    </row>
-    <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A19" s="7" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+    </row>
+    <row r="20" ht="150" customHeight="1">
+      <c r="A20" s="9" t="n"/>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+    </row>
+    <row r="21" ht="150" customHeight="1">
+      <c r="A21" s="7" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>NOTE: If these steps don't fix it, or the same error keeps coming back, stop the line and call your lead or mechanic. Do not change machine settings.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="A21:D21"/>
+  <mergeCells count="4">
+    <mergeCell ref="A2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A4:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>